<commit_message>
Add dashboard and unit price
</commit_message>
<xml_diff>
--- a/Dummy Data/3-March/Upload/Service1/Service1-1.xlsx
+++ b/Dummy Data/3-March/Upload/Service1/Service1-1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elyas/Desktop/NUS/Internship/programs/202X/1-January/Upload/Service1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elyas/Desktop/NUS/Internship/programs/Dummy Data/3-March/Upload/Service1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99629472-1082-CA4E-B5B4-F7D0800F4F61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A65903-0CC0-9F4E-87D9-6DBF44777AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{1FB9A1EF-FA42-E74B-AB40-F96FB4DE8284}"/>
   </bookViews>
@@ -525,7 +525,7 @@
         <v>104444</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G4">
         <v>10003</v>

</xml_diff>